<commit_message>
📊 Deploy Selenium E2E Reports — Build #2 2fc69e376d1558b77f7516ed34e4927a29622489
</commit_message>
<xml_diff>
--- a/reports/latest/reports/Excel/POPC_Selenium_Test_Report.xlsx
+++ b/reports/latest/reports/Excel/POPC_Selenium_Test_Report.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="193">
   <si>
     <t>Test ID</t>
   </si>
@@ -61,7 +61,7 @@
     <t/>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.650Z</t>
+    <t>2026-07-29T12:27:00.433Z</t>
   </si>
   <si>
     <t>TC_PATIENT_002</t>
@@ -76,7 +76,7 @@
     <t>TC_PATIENT_003 — Patient management scenario 3</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.651Z</t>
+    <t>2026-07-29T12:27:00.434Z</t>
   </si>
   <si>
     <t>TC_PATIENT_004</t>
@@ -91,7 +91,7 @@
     <t>TC_PATIENT_005 — Patient management scenario 5</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.652Z</t>
+    <t>2026-07-29T12:27:00.435Z</t>
   </si>
   <si>
     <t>TC_PATIENT_006</t>
@@ -106,7 +106,7 @@
     <t>TC_PATIENT_007 — Patient management scenario 7</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.653Z</t>
+    <t>2026-07-29T12:27:00.436Z</t>
   </si>
   <si>
     <t>TC_PATIENT_008</t>
@@ -115,54 +115,51 @@
     <t>TC_PATIENT_008 — Patient management scenario 8</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.654Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_009</t>
   </si>
   <si>
     <t>TC_PATIENT_009 — Patient management scenario 9</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.437Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_010</t>
   </si>
   <si>
     <t>TC_PATIENT_010 — Patient management scenario 10</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.655Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_011</t>
   </si>
   <si>
     <t>TC_PATIENT_011 — Patient management scenario 11</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.438Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_012</t>
   </si>
   <si>
     <t>TC_PATIENT_012 — Patient management scenario 12</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.656Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_013</t>
   </si>
   <si>
     <t>TC_PATIENT_013 — Patient management scenario 13</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.439Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_014</t>
   </si>
   <si>
     <t>TC_PATIENT_014 — Patient management scenario 14</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.657Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_015</t>
   </si>
   <si>
@@ -175,30 +172,30 @@
     <t>TC_PATIENT_016 — Patient management scenario 16</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.440Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_017</t>
   </si>
   <si>
     <t>TC_PATIENT_017 — Patient management scenario 17</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.658Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_018</t>
   </si>
   <si>
     <t>TC_PATIENT_018 — Patient management scenario 18</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.441Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_019</t>
   </si>
   <si>
     <t>TC_PATIENT_019 — Patient management scenario 19</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.659Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_020</t>
   </si>
   <si>
@@ -211,21 +208,24 @@
     <t>TC_PATIENT_021 — Patient management scenario 21</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.442Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_022</t>
   </si>
   <si>
     <t>TC_PATIENT_022 — Patient management scenario 22</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.660Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_023</t>
   </si>
   <si>
     <t>TC_PATIENT_023 — Patient management scenario 23</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.443Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_024</t>
   </si>
   <si>
@@ -238,24 +238,21 @@
     <t>TC_PATIENT_025 — Patient management scenario 25</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.661Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_026</t>
   </si>
   <si>
     <t>TC_PATIENT_026 — Patient management scenario 26</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.444Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_027</t>
   </si>
   <si>
     <t>TC_PATIENT_027 — Patient management scenario 27</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.662Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_028</t>
   </si>
   <si>
@@ -268,30 +265,30 @@
     <t>TC_PATIENT_029 — Patient management scenario 29</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.445Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_030</t>
   </si>
   <si>
     <t>TC_PATIENT_030 — Patient management scenario 30</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.663Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_031</t>
   </si>
   <si>
     <t>TC_PATIENT_031 — Patient management scenario 31</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.446Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_032</t>
   </si>
   <si>
     <t>TC_PATIENT_032 — Patient management scenario 32</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.664Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_033</t>
   </si>
   <si>
@@ -304,7 +301,7 @@
     <t>TC_PATIENT_034 — Patient management scenario 34</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.665Z</t>
+    <t>2026-07-29T12:27:00.447Z</t>
   </si>
   <si>
     <t>TC_PATIENT_035</t>
@@ -319,30 +316,30 @@
     <t>TC_PATIENT_036 — Patient management scenario 36</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.448Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_037</t>
   </si>
   <si>
     <t>TC_PATIENT_037 — Patient management scenario 37</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.666Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_038</t>
   </si>
   <si>
     <t>TC_PATIENT_038 — Patient management scenario 38</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.449Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_039</t>
   </si>
   <si>
     <t>TC_PATIENT_039 — Patient management scenario 39</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.667Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_040</t>
   </si>
   <si>
@@ -355,15 +352,15 @@
     <t>TC_PATIENT_041 — Patient management scenario 41</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.450Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_042</t>
   </si>
   <si>
     <t>TC_PATIENT_042 — Patient management scenario 42</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.668Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_043</t>
   </si>
   <si>
@@ -376,7 +373,7 @@
     <t>TC_PATIENT_044 — Patient management scenario 44</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.669Z</t>
+    <t>2026-07-29T12:27:00.451Z</t>
   </si>
   <si>
     <t>TC_PATIENT_045</t>
@@ -391,15 +388,15 @@
     <t>TC_PATIENT_046 — Patient management scenario 46</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.452Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_047</t>
   </si>
   <si>
     <t>TC_PATIENT_047 — Patient management scenario 47</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.670Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_048</t>
   </si>
   <si>
@@ -412,7 +409,7 @@
     <t>TC_PATIENT_049 — Patient management scenario 49</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.671Z</t>
+    <t>2026-07-29T12:27:00.453Z</t>
   </si>
   <si>
     <t>TC_PATIENT_050</t>
@@ -427,30 +424,30 @@
     <t>TC_PATIENT_051 — Patient management scenario 51</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.454Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_052</t>
   </si>
   <si>
     <t>TC_PATIENT_052 — Patient management scenario 52</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.672Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_053</t>
   </si>
   <si>
     <t>TC_PATIENT_053 — Patient management scenario 53</t>
   </si>
   <si>
+    <t>2026-07-29T12:27:00.455Z</t>
+  </si>
+  <si>
     <t>TC_PATIENT_054</t>
   </si>
   <si>
     <t>TC_PATIENT_054 — Patient management scenario 54</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.673Z</t>
-  </si>
-  <si>
     <t>TC_PATIENT_055</t>
   </si>
   <si>
@@ -463,7 +460,7 @@
     <t>TC_PATIENT_056 — Patient management scenario 56</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.674Z</t>
+    <t>2026-07-29T12:27:00.456Z</t>
   </si>
   <si>
     <t>TC_PATIENT_057</t>
@@ -484,7 +481,7 @@
     <t>TC_PATIENT_059 — Patient management scenario 59</t>
   </si>
   <si>
-    <t>2026-07-29T11:42:26.675Z</t>
+    <t>2026-07-29T12:27:00.457Z</t>
   </si>
   <si>
     <t>TC_PATIENT_060</t>
@@ -541,13 +538,13 @@
     <t>Session Start</t>
   </si>
   <si>
-    <t>2026-07-29T11:43:11.899Z</t>
+    <t>2026-07-29T12:27:31.117Z</t>
   </si>
   <si>
     <t>Session End</t>
   </si>
   <si>
-    <t>2026-07-29T11:43:11.933Z</t>
+    <t>2026-07-29T12:27:31.150Z</t>
   </si>
   <si>
     <t>Framework</t>
@@ -577,7 +574,7 @@
     <t>Report Generated</t>
   </si>
   <si>
-    <t>2026-07-29T11:43:11.938Z</t>
+    <t>2026-07-29T12:27:31.154Z</t>
   </si>
   <si>
     <t>Total Tests</t>
@@ -1157,7 +1154,7 @@
         <v>12</v>
       </c>
       <c r="F2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -1209,7 +1206,7 @@
         <v>12</v>
       </c>
       <c r="F4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -1345,33 +1342,33 @@
         <v>13</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1397,33 +1394,33 @@
         <v>13</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="2">
+        <v>1</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="2">
-        <v>0</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1449,33 +1446,33 @@
         <v>13</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="2">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1501,19 +1498,19 @@
         <v>13</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="D16" s="2" t="s">
         <v>11</v>
       </c>
@@ -1527,33 +1524,33 @@
         <v>13</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="4">
+        <v>0</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="4">
-        <v>0</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1579,33 +1576,33 @@
         <v>13</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="4">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H19" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="4">
-        <v>0</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1631,19 +1628,19 @@
         <v>13</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>61</v>
-      </c>
       <c r="D21" s="4" t="s">
         <v>11</v>
       </c>
@@ -1657,33 +1654,33 @@
         <v>13</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="2">
+        <v>0</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F22" s="2">
-        <v>0</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1709,33 +1706,33 @@
         <v>13</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F24" s="2">
-        <v>0</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1761,7 +1758,7 @@
         <v>13</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1787,33 +1784,33 @@
         <v>13</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" s="4" t="s">
+      <c r="D27" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" s="4">
+        <v>0</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F27" s="4">
-        <v>0</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1833,25 +1830,25 @@
         <v>12</v>
       </c>
       <c r="F28" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>80</v>
-      </c>
       <c r="D29" s="4" t="s">
         <v>11</v>
       </c>
@@ -1865,33 +1862,33 @@
         <v>13</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F30" s="2">
-        <v>0</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1917,33 +1914,33 @@
         <v>13</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F32" s="2">
+        <v>1</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F32" s="2">
-        <v>0</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1969,19 +1966,19 @@
         <v>13</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="D34" s="2" t="s">
         <v>11</v>
       </c>
@@ -1995,45 +1992,45 @@
         <v>13</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" s="4" t="s">
+      <c r="D35" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" s="4">
+        <v>0</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H35" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F35" s="4">
-        <v>0</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H35" s="4" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="D36" s="2" t="s">
         <v>11</v>
       </c>
@@ -2047,33 +2044,33 @@
         <v>13</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" s="4" t="s">
+      <c r="D37" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37" s="4">
+        <v>1</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H37" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F37" s="4">
-        <v>0</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H37" s="4" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2099,33 +2096,33 @@
         <v>13</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C39" s="4" t="s">
+      <c r="D39" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F39" s="4">
+        <v>1</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H39" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F39" s="4">
-        <v>0</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H39" s="4" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2145,25 +2142,25 @@
         <v>12</v>
       </c>
       <c r="F40" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>13</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>109</v>
-      </c>
       <c r="D41" s="4" t="s">
         <v>11</v>
       </c>
@@ -2177,33 +2174,33 @@
         <v>13</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C42" s="2" t="s">
+      <c r="D42" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F42" s="2">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H42" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F42" s="2">
-        <v>0</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2229,19 +2226,19 @@
         <v>13</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>116</v>
-      </c>
       <c r="D44" s="2" t="s">
         <v>11</v>
       </c>
@@ -2255,45 +2252,45 @@
         <v>13</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C45" s="4" t="s">
+      <c r="D45" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F45" s="4">
+        <v>0</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H45" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E45" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F45" s="4">
-        <v>1</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H45" s="4" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>121</v>
-      </c>
       <c r="D46" s="2" t="s">
         <v>11</v>
       </c>
@@ -2307,33 +2304,33 @@
         <v>13</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C47" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B47" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C47" s="4" t="s">
+      <c r="D47" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F47" s="4">
+        <v>0</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H47" s="4" t="s">
         <v>123</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E47" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F47" s="4">
-        <v>0</v>
-      </c>
-      <c r="G47" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H47" s="4" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2359,19 +2356,19 @@
         <v>13</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>128</v>
-      </c>
       <c r="D49" s="4" t="s">
         <v>11</v>
       </c>
@@ -2385,45 +2382,45 @@
         <v>13</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C50" s="2" t="s">
+      <c r="D50" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F50" s="2">
+        <v>0</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H50" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F50" s="2">
-        <v>0</v>
-      </c>
-      <c r="G50" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C51" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="D51" s="4" t="s">
         <v>11</v>
       </c>
@@ -2437,33 +2434,33 @@
         <v>13</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C52" s="2" t="s">
+      <c r="D52" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F52" s="2">
+        <v>1</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H52" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E52" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F52" s="2">
-        <v>0</v>
-      </c>
-      <c r="G52" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H52" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2489,33 +2486,33 @@
         <v>13</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C54" s="2" t="s">
+      <c r="D54" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F54" s="2">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H54" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F54" s="2">
-        <v>0</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2541,19 +2538,19 @@
         <v>13</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="D56" s="2" t="s">
         <v>11</v>
       </c>
@@ -2567,45 +2564,45 @@
         <v>13</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C57" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C57" s="4" t="s">
+      <c r="D57" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F57" s="4">
+        <v>0</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H57" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F57" s="4">
-        <v>0</v>
-      </c>
-      <c r="G57" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="H57" s="4" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="D58" s="2" t="s">
         <v>11</v>
       </c>
@@ -2619,19 +2616,19 @@
         <v>13</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B59" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>152</v>
-      </c>
       <c r="D59" s="4" t="s">
         <v>11</v>
       </c>
@@ -2645,45 +2642,45 @@
         <v>13</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C60" s="2" t="s">
+      <c r="D60" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F60" s="2">
+        <v>0</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H60" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E60" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F60" s="2">
-        <v>0</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B61" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>157</v>
-      </c>
       <c r="D61" s="4" t="s">
         <v>11</v>
       </c>
@@ -2697,7 +2694,7 @@
         <v>13</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -2750,7 +2747,7 @@
         <v>10</v>
       </c>
       <c r="D2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>14</v>
@@ -2784,7 +2781,7 @@
         <v>18</v>
       </c>
       <c r="D4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>19</v>
@@ -2872,24 +2869,24 @@
         <v>0</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="D10" s="2">
-        <v>0</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2906,24 +2903,24 @@
         <v>0</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D12" s="2">
-        <v>0</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2940,24 +2937,24 @@
         <v>0</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="D14" s="2">
-        <v>0</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -2974,41 +2971,41 @@
         <v>0</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="D16" s="2">
         <v>0</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="4">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="D17" s="4">
-        <v>0</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3025,24 +3022,24 @@
         <v>0</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="4">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="D19" s="4">
-        <v>0</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3059,41 +3056,41 @@
         <v>0</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>61</v>
-      </c>
       <c r="D21" s="4">
         <v>0</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2">
+        <v>0</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="D22" s="2">
-        <v>0</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3110,24 +3107,24 @@
         <v>0</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D24" s="2">
-        <v>0</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3144,7 +3141,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3161,24 +3158,24 @@
         <v>0</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" s="4" t="s">
+      <c r="D27" s="4">
+        <v>0</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="D27" s="4">
-        <v>0</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3192,44 +3189,44 @@
         <v>77</v>
       </c>
       <c r="D28" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>80</v>
-      </c>
       <c r="D29" s="4">
         <v>0</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2">
+        <v>0</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="D30" s="2">
-        <v>0</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3246,24 +3243,24 @@
         <v>0</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="D32" s="2">
-        <v>0</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3280,75 +3277,75 @@
         <v>0</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="D34" s="2">
         <v>0</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" s="4" t="s">
+      <c r="D35" s="4">
+        <v>0</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="D35" s="4">
-        <v>0</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="D36" s="2">
         <v>0</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" s="4" t="s">
+      <c r="D37" s="4">
+        <v>1</v>
+      </c>
+      <c r="E37" s="4" t="s">
         <v>99</v>
-      </c>
-      <c r="D37" s="4">
-        <v>0</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3365,24 +3362,24 @@
         <v>0</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C39" s="4" t="s">
+      <c r="D39" s="4">
+        <v>1</v>
+      </c>
+      <c r="E39" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="D39" s="4">
-        <v>0</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3396,44 +3393,44 @@
         <v>106</v>
       </c>
       <c r="D40" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>109</v>
-      </c>
       <c r="D41" s="4">
         <v>0</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C42" s="2" t="s">
+      <c r="D42" s="2">
+        <v>0</v>
+      </c>
+      <c r="E42" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="D42" s="2">
-        <v>0</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3450,75 +3447,75 @@
         <v>0</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>116</v>
-      </c>
       <c r="D44" s="2">
         <v>0</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C45" s="4" t="s">
+      <c r="D45" s="4">
+        <v>0</v>
+      </c>
+      <c r="E45" s="4" t="s">
         <v>118</v>
-      </c>
-      <c r="D45" s="4">
-        <v>1</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>121</v>
-      </c>
       <c r="D46" s="2">
         <v>0</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C47" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B47" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C47" s="4" t="s">
+      <c r="D47" s="4">
+        <v>0</v>
+      </c>
+      <c r="E47" s="4" t="s">
         <v>123</v>
-      </c>
-      <c r="D47" s="4">
-        <v>0</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3535,75 +3532,75 @@
         <v>0</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>128</v>
-      </c>
       <c r="D49" s="4">
         <v>0</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C50" s="2" t="s">
+      <c r="D50" s="2">
+        <v>0</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="D50" s="2">
-        <v>0</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C51" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>133</v>
-      </c>
       <c r="D51" s="4">
         <v>0</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C52" s="2" t="s">
+      <c r="D52" s="2">
+        <v>1</v>
+      </c>
+      <c r="E52" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="D52" s="2">
-        <v>0</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3620,24 +3617,24 @@
         <v>0</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C54" s="2" t="s">
+      <c r="D54" s="2">
+        <v>0</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="D54" s="2">
-        <v>0</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3654,109 +3651,109 @@
         <v>0</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="D56" s="2">
         <v>0</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C57" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C57" s="4" t="s">
+      <c r="D57" s="4">
+        <v>0</v>
+      </c>
+      <c r="E57" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="D57" s="4">
-        <v>0</v>
-      </c>
-      <c r="E57" s="4" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="D58" s="2">
         <v>0</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="B59" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>152</v>
-      </c>
       <c r="D59" s="4">
         <v>0</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C60" s="2" t="s">
+      <c r="D60" s="2">
+        <v>0</v>
+      </c>
+      <c r="E60" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="D60" s="2">
-        <v>0</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="B61" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>157</v>
-      </c>
       <c r="D61" s="4">
         <v>0</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -3793,7 +3790,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>5</v>
@@ -3856,15 +3853,15 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>159</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B2" s="2">
         <v>60</v>
@@ -3872,7 +3869,7 @@
     </row>
     <row r="3" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B3" s="4">
         <v>60</v>
@@ -3880,7 +3877,7 @@
     </row>
     <row r="4" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B4" s="2">
         <v>60</v>
@@ -3888,7 +3885,7 @@
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B5" s="4">
         <v>0</v>
@@ -3896,7 +3893,7 @@
     </row>
     <row r="6" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B6" s="2">
         <v>0</v>
@@ -3904,7 +3901,7 @@
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B7" s="4">
         <v>0</v>
@@ -3912,82 +3909,82 @@
     </row>
     <row r="8" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>169</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>173</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>177</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>179</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>181</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>185</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -4013,13 +4010,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D1" s="11" t="s">
         <v>188</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4033,7 +4030,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -4059,13 +4056,13 @@
         <v>1</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C1" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="D1" s="12" t="s">
         <v>191</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4079,7 +4076,7 @@
         <v>60</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>